<commit_message>
Testversie (SALDOPLAN_TESTMODUS=1): inlogcode op het scherm en nooit mailen, balk 'Testversie' op elke pagina, starten met voorbeeldgegevens of leeg, koppelingen in proefmodus, AI netjes uit; nooit aan op app.saldoplan.nl (test). Functies in fra1.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/uit/test.xlsx
+++ b/test/uit/test.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="116">
   <si>
     <t>Datum</t>
   </si>
@@ -183,6 +183,12 @@
     <t>WOmzNopOlv</t>
   </si>
   <si>
+    <t>Omzet EU (verlegd)</t>
+  </si>
+  <si>
+    <t>WOmzNopOlb</t>
+  </si>
+  <si>
     <t>Totaal omzet</t>
   </si>
   <si>
@@ -219,13 +225,13 @@
     <t>Bank Zakelijk</t>
   </si>
   <si>
-    <t>Ondernemingsvermogen</t>
-  </si>
-  <si>
-    <t>Debiteuren (open facturen)</t>
-  </si>
-  <si>
-    <t>Materiële vaste activa (boekwaarde)</t>
+    <t>Eigen geld in je bedrijf</t>
+  </si>
+  <si>
+    <t>Nog te ontvangen van klanten</t>
+  </si>
+  <si>
+    <t>Spullen voor je bedrijf (waarde nu)</t>
   </si>
   <si>
     <t>Rubriek</t>
@@ -1137,7 +1143,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1178,95 +1184,109 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="7">
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="2">
         <v>1000</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="D4" s="2">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C5" s="7">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="C7" s="2">
-        <v>480</v>
-      </c>
-      <c r="D7" s="2">
-        <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2">
-        <v>100</v>
+        <v>480</v>
       </c>
       <c r="D8" s="2">
-        <v>100</v>
+        <v>480</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C9" s="2">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D9" s="2">
-        <v>48</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="2">
+        <v>60</v>
+      </c>
+      <c r="D10" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>32</v>
       </c>
-      <c r="B10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" s="2">
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="2">
         <v>24.2</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D11" s="2">
         <v>24.2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" s="7">
+    <row r="12" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="7">
         <v>664.2</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D12" s="7">
         <v>652.2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C13" s="7">
-        <v>335.8</v>
-      </c>
-      <c r="D13" s="7">
-        <v>347.8</v>
+    <row r="14" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="7">
+        <v>1335.8</v>
+      </c>
+      <c r="D14" s="7">
+        <v>1347.8</v>
       </c>
     </row>
   </sheetData>
@@ -1288,13 +1308,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>4</v>
@@ -1302,13 +1322,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2">
         <v>954.8</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2">
         <v>3874.8</v>
@@ -1316,7 +1336,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B3" s="2">
         <v>1000</v>
@@ -1327,7 +1347,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" s="2">
         <v>1920</v>
@@ -1367,27 +1387,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="2">
         <v>1000</v>
@@ -1407,7 +1427,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="2">
         <v>210</v>
@@ -1427,7 +1447,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B4" s="2">
         <v>0</v>
@@ -1447,7 +1467,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -1467,7 +1487,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -1487,7 +1507,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" s="2">
         <v>0</v>
@@ -1507,7 +1527,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B8" s="2">
         <v>0</v>
@@ -1527,7 +1547,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B9" s="2">
         <v>0</v>
@@ -1547,7 +1567,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B10" s="2">
         <v>0</v>
@@ -1567,7 +1587,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B11" s="2">
         <v>0</v>
@@ -1587,13 +1607,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B12" s="2">
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
@@ -1602,12 +1622,12 @@
         <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B13" s="2">
         <v>0</v>
@@ -1627,7 +1647,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B14" s="2">
         <v>0</v>
@@ -1647,7 +1667,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B15" s="2">
         <v>0</v>
@@ -1667,7 +1687,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B16" s="2">
         <v>0</v>
@@ -1687,7 +1707,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B17" s="2">
         <v>210</v>
@@ -1707,7 +1727,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B18" s="2">
         <v>21</v>
@@ -1727,7 +1747,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B19" s="2">
         <v>189</v>
@@ -1771,10 +1791,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>41</v>
@@ -1789,7 +1809,7 @@
         <v>43</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1819,16 +1839,16 @@
         <v>38</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="2:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1863,25 +1883,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1897,31 +1917,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B4">
         <v>2026</v>
@@ -1929,10 +1949,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B5" s="8">
-        <v>46306.96079884259</v>
+        <v>46307.563732870374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Testuitvoer (test/uit) terug naar de vorige versie; hoorde niet in de vorige commit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/uit/test.xlsx
+++ b/test/uit/test.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="114">
   <si>
     <t>Datum</t>
   </si>
@@ -183,12 +183,6 @@
     <t>WOmzNopOlv</t>
   </si>
   <si>
-    <t>Omzet EU (verlegd)</t>
-  </si>
-  <si>
-    <t>WOmzNopOlb</t>
-  </si>
-  <si>
     <t>Totaal omzet</t>
   </si>
   <si>
@@ -225,13 +219,13 @@
     <t>Bank Zakelijk</t>
   </si>
   <si>
-    <t>Eigen geld in je bedrijf</t>
-  </si>
-  <si>
-    <t>Nog te ontvangen van klanten</t>
-  </si>
-  <si>
-    <t>Spullen voor je bedrijf (waarde nu)</t>
+    <t>Ondernemingsvermogen</t>
+  </si>
+  <si>
+    <t>Debiteuren (open facturen)</t>
+  </si>
+  <si>
+    <t>Materiële vaste activa (boekwaarde)</t>
   </si>
   <si>
     <t>Rubriek</t>
@@ -1143,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1184,109 +1178,95 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="7">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="2">
-        <v>1000</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="7">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="B7" t="s">
         <v>57</v>
+      </c>
+      <c r="C7" s="2">
+        <v>480</v>
+      </c>
+      <c r="D7" s="2">
+        <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
         <v>58</v>
       </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
       <c r="C8" s="2">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="D8" s="2">
-        <v>480</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="2">
         <v>60</v>
       </c>
-      <c r="C9" s="2">
-        <v>100</v>
-      </c>
       <c r="D9" s="2">
-        <v>100</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="D10" s="2">
+        <v>24.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="2">
-        <v>60</v>
-      </c>
-      <c r="D10" s="2">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" s="7">
+        <v>664.2</v>
+      </c>
+      <c r="D11" s="7">
+        <v>652.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="2">
-        <v>24.2</v>
-      </c>
-      <c r="D11" s="2">
-        <v>24.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="7">
-        <v>664.2</v>
-      </c>
-      <c r="D12" s="7">
-        <v>652.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14" s="7">
-        <v>1335.8</v>
-      </c>
-      <c r="D14" s="7">
-        <v>1347.8</v>
+      <c r="C13" s="7">
+        <v>335.8</v>
+      </c>
+      <c r="D13" s="7">
+        <v>347.8</v>
       </c>
     </row>
   </sheetData>
@@ -1308,13 +1288,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>4</v>
@@ -1322,13 +1302,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2">
         <v>954.8</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2">
         <v>3874.8</v>
@@ -1336,7 +1316,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B3" s="2">
         <v>1000</v>
@@ -1347,7 +1327,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B4" s="2">
         <v>1920</v>
@@ -1387,27 +1367,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2">
         <v>1000</v>
@@ -1427,7 +1407,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B3" s="2">
         <v>210</v>
@@ -1447,7 +1427,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B4" s="2">
         <v>0</v>
@@ -1467,7 +1447,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -1487,7 +1467,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -1507,7 +1487,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B7" s="2">
         <v>0</v>
@@ -1527,7 +1507,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="2">
         <v>0</v>
@@ -1547,7 +1527,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B9" s="2">
         <v>0</v>
@@ -1567,7 +1547,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B10" s="2">
         <v>0</v>
@@ -1587,7 +1567,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B11" s="2">
         <v>0</v>
@@ -1607,13 +1587,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B12" s="2">
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
@@ -1622,12 +1602,12 @@
         <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B13" s="2">
         <v>0</v>
@@ -1647,7 +1627,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B14" s="2">
         <v>0</v>
@@ -1667,7 +1647,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B15" s="2">
         <v>0</v>
@@ -1687,7 +1667,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B16" s="2">
         <v>0</v>
@@ -1707,7 +1687,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B17" s="2">
         <v>210</v>
@@ -1727,7 +1707,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B18" s="2">
         <v>21</v>
@@ -1747,7 +1727,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B19" s="2">
         <v>189</v>
@@ -1791,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>41</v>
@@ -1809,7 +1789,7 @@
         <v>43</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1839,16 +1819,16 @@
         <v>38</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="2:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1883,25 +1863,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1917,31 +1897,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B4">
         <v>2026</v>
@@ -1949,10 +1929,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B5" s="8">
-        <v>46307.563732870374</v>
+        <v>46306.96079884259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Beheer (/admin) voor Saldoplan zelf: klanten zoeken en bekijken (zonder bankregels), proef verlengen, blokkeren, meekijken met reden (alleen kijken, 1 uur, balk), cijfers uit eigen DB en Stripe-status (aanmeldingen, actief, proef naar betaald, opzeggingen, MRR, AI-gebruik en daglimiet per klant), storingen (dagtaak, koppelingen, mislukte mails) en logboek. Alleen ADMIN_EMAILS met tweestap. Feedbackknop in de app met schermafbeelding, pagina en toestel; optionele webhook. Tests: gewone klant komt er nooit in, acties en meekijken worden gelogd.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/uit/test.xlsx
+++ b/test/uit/test.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="116">
   <si>
     <t>Datum</t>
   </si>
@@ -183,6 +183,12 @@
     <t>WOmzNopOlv</t>
   </si>
   <si>
+    <t>Omzet EU (verlegd)</t>
+  </si>
+  <si>
+    <t>WOmzNopOlb</t>
+  </si>
+  <si>
     <t>Totaal omzet</t>
   </si>
   <si>
@@ -219,13 +225,13 @@
     <t>Bank Zakelijk</t>
   </si>
   <si>
-    <t>Ondernemingsvermogen</t>
-  </si>
-  <si>
-    <t>Debiteuren (open facturen)</t>
-  </si>
-  <si>
-    <t>Materiële vaste activa (boekwaarde)</t>
+    <t>Eigen geld in je bedrijf</t>
+  </si>
+  <si>
+    <t>Nog te ontvangen van klanten</t>
+  </si>
+  <si>
+    <t>Spullen voor je bedrijf (waarde nu)</t>
   </si>
   <si>
     <t>Rubriek</t>
@@ -1137,7 +1143,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1178,95 +1184,109 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="7">
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="2">
         <v>1000</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="D4" s="2">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C5" s="7">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="C7" s="2">
-        <v>480</v>
-      </c>
-      <c r="D7" s="2">
-        <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2">
-        <v>100</v>
+        <v>480</v>
       </c>
       <c r="D8" s="2">
-        <v>100</v>
+        <v>480</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C9" s="2">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D9" s="2">
-        <v>48</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="2">
+        <v>60</v>
+      </c>
+      <c r="D10" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>32</v>
       </c>
-      <c r="B10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" s="2">
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="2">
         <v>24.2</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D11" s="2">
         <v>24.2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" s="7">
+    <row r="12" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="7">
         <v>664.2</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D12" s="7">
         <v>652.2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C13" s="7">
-        <v>335.8</v>
-      </c>
-      <c r="D13" s="7">
-        <v>347.8</v>
+    <row r="14" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="7">
+        <v>1335.8</v>
+      </c>
+      <c r="D14" s="7">
+        <v>1347.8</v>
       </c>
     </row>
   </sheetData>
@@ -1288,13 +1308,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>4</v>
@@ -1302,13 +1322,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2">
         <v>954.8</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2">
         <v>3874.8</v>
@@ -1316,7 +1336,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B3" s="2">
         <v>1000</v>
@@ -1327,7 +1347,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" s="2">
         <v>1920</v>
@@ -1367,27 +1387,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="2">
         <v>1000</v>
@@ -1407,7 +1427,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="2">
         <v>210</v>
@@ -1427,7 +1447,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B4" s="2">
         <v>0</v>
@@ -1447,7 +1467,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -1467,7 +1487,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -1487,7 +1507,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" s="2">
         <v>0</v>
@@ -1507,7 +1527,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B8" s="2">
         <v>0</v>
@@ -1527,7 +1547,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B9" s="2">
         <v>0</v>
@@ -1547,7 +1567,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B10" s="2">
         <v>0</v>
@@ -1567,7 +1587,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B11" s="2">
         <v>0</v>
@@ -1587,13 +1607,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B12" s="2">
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
@@ -1602,12 +1622,12 @@
         <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B13" s="2">
         <v>0</v>
@@ -1627,7 +1647,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B14" s="2">
         <v>0</v>
@@ -1647,7 +1667,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B15" s="2">
         <v>0</v>
@@ -1667,7 +1687,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B16" s="2">
         <v>0</v>
@@ -1687,7 +1707,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B17" s="2">
         <v>210</v>
@@ -1707,7 +1727,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B18" s="2">
         <v>21</v>
@@ -1727,7 +1747,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B19" s="2">
         <v>189</v>
@@ -1771,10 +1791,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>41</v>
@@ -1789,7 +1809,7 @@
         <v>43</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1819,16 +1839,16 @@
         <v>38</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="2:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1863,25 +1883,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1897,31 +1917,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B4">
         <v>2026</v>
@@ -1929,10 +1949,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B5" s="8">
-        <v>46306.96079884259</v>
+        <v>46307.605605543984</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Testuitvoer (test/uit) terug; hoort niet in de commit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/uit/test.xlsx
+++ b/test/uit/test.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="114">
   <si>
     <t>Datum</t>
   </si>
@@ -183,12 +183,6 @@
     <t>WOmzNopOlv</t>
   </si>
   <si>
-    <t>Omzet EU (verlegd)</t>
-  </si>
-  <si>
-    <t>WOmzNopOlb</t>
-  </si>
-  <si>
     <t>Totaal omzet</t>
   </si>
   <si>
@@ -225,13 +219,13 @@
     <t>Bank Zakelijk</t>
   </si>
   <si>
-    <t>Eigen geld in je bedrijf</t>
-  </si>
-  <si>
-    <t>Nog te ontvangen van klanten</t>
-  </si>
-  <si>
-    <t>Spullen voor je bedrijf (waarde nu)</t>
+    <t>Ondernemingsvermogen</t>
+  </si>
+  <si>
+    <t>Debiteuren (open facturen)</t>
+  </si>
+  <si>
+    <t>Materiële vaste activa (boekwaarde)</t>
   </si>
   <si>
     <t>Rubriek</t>
@@ -1143,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1184,109 +1178,95 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="7">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="2">
-        <v>1000</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="7">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="B7" t="s">
         <v>57</v>
+      </c>
+      <c r="C7" s="2">
+        <v>480</v>
+      </c>
+      <c r="D7" s="2">
+        <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
         <v>58</v>
       </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
       <c r="C8" s="2">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="D8" s="2">
-        <v>480</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="2">
         <v>60</v>
       </c>
-      <c r="C9" s="2">
-        <v>100</v>
-      </c>
       <c r="D9" s="2">
-        <v>100</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="D10" s="2">
+        <v>24.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="2">
-        <v>60</v>
-      </c>
-      <c r="D10" s="2">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" s="7">
+        <v>664.2</v>
+      </c>
+      <c r="D11" s="7">
+        <v>652.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="2">
-        <v>24.2</v>
-      </c>
-      <c r="D11" s="2">
-        <v>24.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="7">
-        <v>664.2</v>
-      </c>
-      <c r="D12" s="7">
-        <v>652.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14" s="7">
-        <v>1335.8</v>
-      </c>
-      <c r="D14" s="7">
-        <v>1347.8</v>
+      <c r="C13" s="7">
+        <v>335.8</v>
+      </c>
+      <c r="D13" s="7">
+        <v>347.8</v>
       </c>
     </row>
   </sheetData>
@@ -1308,13 +1288,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>4</v>
@@ -1322,13 +1302,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2">
         <v>954.8</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2">
         <v>3874.8</v>
@@ -1336,7 +1316,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B3" s="2">
         <v>1000</v>
@@ -1347,7 +1327,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B4" s="2">
         <v>1920</v>
@@ -1387,27 +1367,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2">
         <v>1000</v>
@@ -1427,7 +1407,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B3" s="2">
         <v>210</v>
@@ -1447,7 +1427,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B4" s="2">
         <v>0</v>
@@ -1467,7 +1447,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -1487,7 +1467,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -1507,7 +1487,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B7" s="2">
         <v>0</v>
@@ -1527,7 +1507,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="2">
         <v>0</v>
@@ -1547,7 +1527,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B9" s="2">
         <v>0</v>
@@ -1567,7 +1547,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B10" s="2">
         <v>0</v>
@@ -1587,7 +1567,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B11" s="2">
         <v>0</v>
@@ -1607,13 +1587,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B12" s="2">
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
@@ -1622,12 +1602,12 @@
         <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B13" s="2">
         <v>0</v>
@@ -1647,7 +1627,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B14" s="2">
         <v>0</v>
@@ -1667,7 +1647,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B15" s="2">
         <v>0</v>
@@ -1687,7 +1667,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B16" s="2">
         <v>0</v>
@@ -1707,7 +1687,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B17" s="2">
         <v>210</v>
@@ -1727,7 +1707,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B18" s="2">
         <v>21</v>
@@ -1747,7 +1727,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B19" s="2">
         <v>189</v>
@@ -1791,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>41</v>
@@ -1809,7 +1789,7 @@
         <v>43</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1839,16 +1819,16 @@
         <v>38</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="2:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1883,25 +1863,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1917,31 +1897,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B4">
         <v>2026</v>
@@ -1949,10 +1929,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B5" s="8">
-        <v>46307.605605543984</v>
+        <v>46306.96079884259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>